<commit_message>
Fix review findings: W-9 TIN digits, workbook DOB cells, extension bypass
- Regenerate every PDF from its original vector file with row-level
  matching of single-character boxes (W-9 TIN, I-9 SSN comb field) and a
  coverage proof that every original value on a page is redacted before
  the file is written.
- Rewrite original DOB date cells in the "Master Driver Data" sheet,
  whose header sits below a title block.
- Middleware: run on every path except Next.js build assets; treat a
  file-extension path as static only under a real public/ folder; decode
  and collapse paths before the policy check; deny undecodable paths.
- Add the reviewer's bypass cases to route-access tests and the redacted
  round-1 review to docs/security.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018duWUaDT6w9VgbJkw7sny8
</commit_message>
<xml_diff>
--- a/public/data/main-source-v2_enhanced_bof_aligned.xlsx
+++ b/public/data/main-source-v2_enhanced_bof_aligned.xlsx
@@ -44954,7 +44954,7 @@
         <v>358</v>
       </c>
       <c r="N4" s="49">
-        <v>25941</v>
+        <v>25934</v>
       </c>
       <c r="O4" s="48" t="s">
         <v>310</v>
@@ -45056,7 +45056,7 @@
         <v>359</v>
       </c>
       <c r="N5" s="52">
-        <v>30320</v>
+        <v>30317</v>
       </c>
       <c r="O5" s="51" t="s">
         <v>311</v>
@@ -45158,7 +45158,7 @@
         <v>360</v>
       </c>
       <c r="N6" s="49">
-        <v>25937</v>
+        <v>25934</v>
       </c>
       <c r="O6" s="48" t="s">
         <v>310</v>
@@ -45260,7 +45260,7 @@
         <v>358</v>
       </c>
       <c r="N7" s="52">
-        <v>34193</v>
+        <v>33970</v>
       </c>
       <c r="O7" s="51" t="s">
         <v>311</v>
@@ -45362,7 +45362,7 @@
         <v>358</v>
       </c>
       <c r="N8" s="49">
-        <v>24398</v>
+        <v>24108</v>
       </c>
       <c r="O8" s="48" t="s">
         <v>310</v>
@@ -45464,7 +45464,7 @@
         <v>361</v>
       </c>
       <c r="N9" s="52">
-        <v>25607</v>
+        <v>25569</v>
       </c>
       <c r="O9" s="51" t="s">
         <v>310</v>
@@ -45566,7 +45566,7 @@
         <v>358</v>
       </c>
       <c r="N10" s="49">
-        <v>36508</v>
+        <v>36161</v>
       </c>
       <c r="O10" s="48" t="s">
         <v>311</v>
@@ -45668,7 +45668,7 @@
         <v>358</v>
       </c>
       <c r="N11" s="52">
-        <v>23612</v>
+        <v>23377</v>
       </c>
       <c r="O11" s="51" t="s">
         <v>310</v>
@@ -45770,7 +45770,7 @@
         <v>358</v>
       </c>
       <c r="N12" s="49">
-        <v>30971</v>
+        <v>30682</v>
       </c>
       <c r="O12" s="48" t="s">
         <v>311</v>
@@ -45872,7 +45872,7 @@
         <v>359</v>
       </c>
       <c r="N13" s="52">
-        <v>24361</v>
+        <v>24108</v>
       </c>
       <c r="O13" s="51" t="s">
         <v>310</v>
@@ -45974,7 +45974,7 @@
         <v>360</v>
       </c>
       <c r="N14" s="49">
-        <v>24911</v>
+        <v>24838</v>
       </c>
       <c r="O14" s="48" t="s">
         <v>311</v>
@@ -46076,7 +46076,7 @@
         <v>359</v>
       </c>
       <c r="N15" s="52">
-        <v>32974</v>
+        <v>32874</v>
       </c>
       <c r="O15" s="51" t="s">
         <v>310</v>

</xml_diff>